<commit_message>
fix: use the sum of the five cited Dallas tax components, 2.226710, as the property tax rate
</commit_message>
<xml_diff>
--- a/docs/proforma-reference.xlsx
+++ b/docs/proforma-reference.xlsx
@@ -1481,11 +1481,11 @@
       </c>
       <c r="D2" s="2" t="n">
         <f aca="false">S1!B52</f>
-        <v>1313240.26</v>
+        <v>1313239.71</v>
       </c>
       <c r="E2" s="2" t="n">
         <f aca="false">S1!B53</f>
-        <v>107559.59</v>
+        <v>107560.14</v>
       </c>
       <c r="F2" s="3" t="n">
         <f aca="false">S1!B54</f>
@@ -1501,11 +1501,11 @@
       </c>
       <c r="I2" s="2" t="n">
         <f aca="false">S1!B61</f>
-        <v>324271.11</v>
+        <v>324271.5</v>
       </c>
       <c r="J2" s="2" t="n">
         <f aca="false">S1!B62</f>
-        <v>-95728.89</v>
+        <v>-95728.5</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1522,11 +1522,11 @@
       </c>
       <c r="D3" s="2" t="n">
         <f aca="false">S2!B46</f>
-        <v>1251174.33</v>
+        <v>1251173.94</v>
       </c>
       <c r="E3" s="2" t="n">
         <f aca="false">S2!B47</f>
-        <v>238226.17</v>
+        <v>238226.56</v>
       </c>
       <c r="F3" s="3" t="n">
         <f aca="false">S2!B48</f>
@@ -1542,11 +1542,11 @@
       </c>
       <c r="I3" s="2" t="n">
         <f aca="false">S2!B55</f>
-        <v>313436.17</v>
+        <v>313436.54</v>
       </c>
       <c r="J3" s="2" t="n">
         <f aca="false">S2!B56</f>
-        <v>13436.17</v>
+        <v>13436.54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1563,11 +1563,11 @@
       </c>
       <c r="D4" s="2" t="n">
         <f aca="false">S3!B46</f>
-        <v>1191258.52</v>
+        <v>1191257.87</v>
       </c>
       <c r="E4" s="2" t="n">
         <f aca="false">S3!B47</f>
-        <v>-512840.76</v>
+        <v>-512840.11</v>
       </c>
       <c r="F4" s="3" t="n">
         <f aca="false">S3!B48</f>
@@ -1830,7 +1830,7 @@
         <v>59</v>
       </c>
       <c r="B16" s="0" t="n">
-        <v>2.226885</v>
+        <v>2.22671</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>60</v>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="E31" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),ROUND($B$61*Assumptions!$B$2/100,2),"")</f>
-        <v>3242.71</v>
+        <v>3242.72</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>184</v>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="E38" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),$B$61+E32+E33+E34+E35,"")</f>
-        <v>1040217.51</v>
+        <v>1040217.9</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>212</v>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="E39" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),ROUND(E38*Assumptions!$B$10/100,2),"")</f>
-        <v>832174.01</v>
+        <v>832174.32</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>216</v>
@@ -2759,7 +2759,7 @@
       </c>
       <c r="E40" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),ROUND(($B$61+E32+E35)*Assumptions!$B$10/100*Assumptions!$B$11/100/12*Assumptions!$B$15,2),"")</f>
-        <v>24492.09</v>
+        <v>24492.11</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>220</v>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="E42" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),E40+E41,"")</f>
-        <v>49140.71</v>
+        <v>49140.73</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>228</v>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="E43" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),ROUND(E39*Assumptions!$B$12/100,2),"")</f>
-        <v>16643.48</v>
+        <v>16643.49</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>232</v>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="E45" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),E42+E43+E44,"")</f>
-        <v>66784.19</v>
+        <v>66784.22</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>240</v>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="B46" s="2" t="n">
         <f aca="false">ROUND(B2*Assumptions!$B$16/100*Assumptions!$B$15/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>242</v>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="E46" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),ROUND($B$61*Assumptions!$B$16/100*Assumptions!$B$15/12,2),"")</f>
-        <v>5415.86</v>
+        <v>5415.44</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>244</v>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="B48" s="2" t="n">
         <f aca="false">B46+B47</f>
-        <v>13786.29</v>
+        <v>13785.74</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>250</v>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="E48" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),E46+E47,"")</f>
-        <v>12187.46</v>
+        <v>12187.04</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>252</v>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="B52" s="2" t="n">
         <f aca="false">B2+B31+B32+B33+B34+B35+B45+B48+B51</f>
-        <v>1313240.26</v>
+        <v>1313239.71</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>265</v>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="E52" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),$B$61+E31+E32+E33+E34+E35+E45+E48+E51,"")</f>
-        <v>1207679.86</v>
+        <v>1207679.87</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>267</v>
@@ -3035,7 +3035,7 @@
       </c>
       <c r="B53" s="2" t="n">
         <f aca="false">B30-B52</f>
-        <v>107559.59</v>
+        <v>107560.14</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>268</v>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="E53" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),B30-E52,"")</f>
-        <v>213119.99</v>
+        <v>213119.98</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>270</v>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="B55" s="2" t="n">
         <f aca="false">B52-B51-B39</f>
-        <v>319235.15</v>
+        <v>319234.6</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>275</v>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="E55" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$61),E52-E51-E39,"")</f>
-        <v>290257.86</v>
+        <v>290257.56</v>
       </c>
       <c r="F55" s="4" t="s">
         <v>277</v>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="B59" s="11" t="n">
         <f aca="false">1+Assumptions!$B$2/100+Assumptions!$B$10/100*(Assumptions!$B$12/100+Assumptions!$B$11/100/12*Assumptions!$B$15)+(Assumptions!$B$16/100)*Assumptions!$B$15/12</f>
-        <v>1.1027016375</v>
+        <v>1.102700325</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>288</v>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="B61" s="2" t="n">
         <f aca="false">IF(B60&lt;0,"none",ROUNDDOWN(B60/B59,2))</f>
-        <v>324271.11</v>
+        <v>324271.5</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>294</v>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="B62" s="2" t="n">
         <f aca="false">IF(ISNUMBER(B61),B61-B2,"")</f>
-        <v>-95728.89</v>
+        <v>-95728.5</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>297</v>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="B64" s="2" t="n">
         <f aca="false">IF(ISNUMBER(B61),E53,"")</f>
-        <v>213119.99</v>
+        <v>213119.98</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>303</v>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="E25" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),ROUND($B$55*Assumptions!$B$2/100,2),"")</f>
-        <v>3134.36</v>
+        <v>3134.37</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>184</v>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="E32" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),$B$55+E26+E27+E28+E29,"")</f>
-        <v>1091486.17</v>
+        <v>1091486.54</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>212</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="E33" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),ROUND(E32*Assumptions!$B$10/100,2),"")</f>
-        <v>873188.94</v>
+        <v>873189.23</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>216</v>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="E34" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),ROUND(($B$55+E26+E29)*Assumptions!$B$10/100*Assumptions!$B$11/100/12*Assumptions!$B$15,2),"")</f>
-        <v>23594.17</v>
+        <v>23594.19</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>220</v>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="E36" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),E34+E35,"")</f>
-        <v>50825.92</v>
+        <v>50825.94</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>228</v>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="E39" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),E36+E37+E38,"")</f>
-        <v>69289.7</v>
+        <v>69289.72</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>240</v>
@@ -3978,7 +3978,7 @@
       </c>
       <c r="B40" s="2" t="n">
         <f aca="false">ROUND(B2*Assumptions!$B$16/100*Assumptions!$B$15/12,2)</f>
-        <v>5010.49</v>
+        <v>5010.1</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>242</v>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="E40" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),ROUND($B$55*Assumptions!$B$16/100*Assumptions!$B$15/12,2),"")</f>
-        <v>5234.9</v>
+        <v>5234.49</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>244</v>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="B42" s="2" t="n">
         <f aca="false">B40+B41</f>
-        <v>12491.74</v>
+        <v>12491.35</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>250</v>
@@ -4032,7 +4032,7 @@
       </c>
       <c r="E42" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),E40+E41,"")</f>
-        <v>12716.15</v>
+        <v>12715.74</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>252</v>
@@ -4110,7 +4110,7 @@
       </c>
       <c r="B46" s="2" t="n">
         <f aca="false">B2+B25+B26+B27+B28+B29+B39+B42+B45</f>
-        <v>1251174.33</v>
+        <v>1251173.94</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>265</v>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="E46" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),$B$55+E25+E26+E27+E28+E29+E39+E42+E45,"")</f>
-        <v>1265990.42</v>
+        <v>1265990.41</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>267</v>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="B47" s="2" t="n">
         <f aca="false">B24-B46</f>
-        <v>238226.17</v>
+        <v>238226.56</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>268</v>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="E47" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),B24-E46,"")</f>
-        <v>223410.08</v>
+        <v>223410.09</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>270</v>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="B49" s="2" t="n">
         <f aca="false">B46-B45-B33</f>
-        <v>299370.29</v>
+        <v>299369.9</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>275</v>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="E49" s="2" t="n">
         <f aca="false">IF(ISNUMBER($B$55),E46-E45-E33,"")</f>
-        <v>303437.44</v>
+        <v>303437.14</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>277</v>
@@ -4257,7 +4257,7 @@
       </c>
       <c r="B53" s="11" t="n">
         <f aca="false">1+Assumptions!$B$2/100+Assumptions!$B$10/100*(Assumptions!$B$12/100+Assumptions!$B$11/100/12*Assumptions!$B$15)+(Assumptions!$B$16/100)*Assumptions!$B$15/12</f>
-        <v>1.1027016375</v>
+        <v>1.102700325</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>288</v>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="B55" s="2" t="n">
         <f aca="false">IF(B54&lt;0,"none",ROUNDDOWN(B54/B53,2))</f>
-        <v>313436.17</v>
+        <v>313436.54</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>294</v>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="B56" s="2" t="n">
         <f aca="false">IF(ISNUMBER(B55),B55-B2,"")</f>
-        <v>13436.17</v>
+        <v>13436.54</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>297</v>
@@ -4332,7 +4332,7 @@
       </c>
       <c r="B58" s="2" t="n">
         <f aca="false">IF(ISNUMBER(B55),E47,"")</f>
-        <v>223410.08</v>
+        <v>223410.09</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>303</v>
@@ -5075,7 +5075,7 @@
       </c>
       <c r="B40" s="2" t="n">
         <f aca="false">ROUND(B2*Assumptions!$B$16/100*Assumptions!$B$15/12,2)</f>
-        <v>8267.31</v>
+        <v>8266.66</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>242</v>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="B42" s="2" t="n">
         <f aca="false">B40+B41</f>
-        <v>13568.31</v>
+        <v>13567.66</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>250</v>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="B46" s="2" t="n">
         <f aca="false">B2+B25+B26+B27+B28+B29+B39+B42+B45</f>
-        <v>1191258.52</v>
+        <v>1191257.87</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>265</v>
@@ -5229,7 +5229,7 @@
       </c>
       <c r="B47" s="2" t="n">
         <f aca="false">B24-B46</f>
-        <v>-512840.76</v>
+        <v>-512840.11</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>268</v>
@@ -5273,7 +5273,7 @@
       </c>
       <c r="B49" s="2" t="n">
         <f aca="false">B46-B45-B33</f>
-        <v>301910.25</v>
+        <v>301909.6</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>275</v>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="B53" s="11" t="n">
         <f aca="false">1+Assumptions!$B$2/100+Assumptions!$B$10/100*(Assumptions!$B$12/100+Assumptions!$B$11/100/12*Assumptions!$B$15)+(Assumptions!$B$16/100)*Assumptions!$B$15/12</f>
-        <v>1.1027016375</v>
+        <v>1.102700325</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>288</v>
@@ -5573,11 +5573,11 @@
       </c>
       <c r="F2" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E2+M2+N2+Y2+AA2+L2</f>
-        <v>1207890.18</v>
+        <v>1207889.81</v>
       </c>
       <c r="G2" s="2" t="n">
         <f aca="false">D2-F2</f>
-        <v>70829.6900000002</v>
+        <v>70830.0600000001</v>
       </c>
       <c r="H2" s="3" t="n">
         <f aca="false">ROUND(G2/D2,4)</f>
@@ -5653,15 +5653,15 @@
       </c>
       <c r="Z2" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C2/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA2" s="2" t="n">
         <f aca="false">Z2+O2</f>
-        <v>8739.42</v>
+        <v>8739.05</v>
       </c>
       <c r="AB2" s="2" t="n">
         <f aca="false">F2-L2-S2</f>
-        <v>278749.58</v>
+        <v>278749.21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5684,11 +5684,11 @@
       </c>
       <c r="F3" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E3+M3+N3+Y3+AA3+L3</f>
-        <v>1229588.63</v>
+        <v>1229588.08</v>
       </c>
       <c r="G3" s="2" t="n">
         <f aca="false">D3-F3</f>
-        <v>49131.2400000002</v>
+        <v>49131.79</v>
       </c>
       <c r="H3" s="3" t="n">
         <f aca="false">ROUND(G3/D3,4)</f>
@@ -5764,15 +5764,15 @@
       </c>
       <c r="Z3" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C3/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA3" s="2" t="n">
         <f aca="false">Z3+O3</f>
-        <v>13109.13</v>
+        <v>13108.58</v>
       </c>
       <c r="AB3" s="2" t="n">
         <f aca="false">F3-L3-S3</f>
-        <v>300448.03</v>
+        <v>300447.48</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5795,11 +5795,11 @@
       </c>
       <c r="F4" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E4+M4+N4+Y4+AA4+L4</f>
-        <v>1251287.08</v>
+        <v>1251286.34</v>
       </c>
       <c r="G4" s="2" t="n">
         <f aca="false">D4-F4</f>
-        <v>27432.79</v>
+        <v>27433.53</v>
       </c>
       <c r="H4" s="3" t="n">
         <f aca="false">ROUND(G4/D4,4)</f>
@@ -5875,15 +5875,15 @@
       </c>
       <c r="Z4" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C4/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA4" s="2" t="n">
         <f aca="false">Z4+O4</f>
-        <v>17478.84</v>
+        <v>17478.1</v>
       </c>
       <c r="AB4" s="2" t="n">
         <f aca="false">F4-L4-S4</f>
-        <v>322146.48</v>
+        <v>322145.74</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5906,11 +5906,11 @@
       </c>
       <c r="F5" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E5+M5+N5+Y5+AA5+L5</f>
-        <v>1281825.23</v>
+        <v>1281824.86</v>
       </c>
       <c r="G5" s="2" t="n">
         <f aca="false">D5-F5</f>
-        <v>-3105.35999999987</v>
+        <v>-3104.98999999976</v>
       </c>
       <c r="H5" s="3" t="n">
         <f aca="false">ROUND(G5/D5,4)</f>
@@ -5986,15 +5986,15 @@
       </c>
       <c r="Z5" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C5/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA5" s="2" t="n">
         <f aca="false">Z5+O5</f>
-        <v>9190.86</v>
+        <v>9190.49</v>
       </c>
       <c r="AB5" s="2" t="n">
         <f aca="false">F5-L5-S5</f>
-        <v>296344.92</v>
+        <v>296344.55</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6017,11 +6017,11 @@
       </c>
       <c r="F6" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E6+M6+N6+Y6+AA6+L6</f>
-        <v>1304715.46</v>
+        <v>1304714.91</v>
       </c>
       <c r="G6" s="2" t="n">
         <f aca="false">D6-F6</f>
-        <v>-25995.5899999999</v>
+        <v>-25995.0399999998</v>
       </c>
       <c r="H6" s="3" t="n">
         <f aca="false">ROUND(G6/D6,4)</f>
@@ -6097,15 +6097,15 @@
       </c>
       <c r="Z6" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C6/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA6" s="2" t="n">
         <f aca="false">Z6+O6</f>
-        <v>13786.29</v>
+        <v>13785.74</v>
       </c>
       <c r="AB6" s="2" t="n">
         <f aca="false">F6-L6-S6</f>
-        <v>319235.15</v>
+        <v>319234.6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6128,11 +6128,11 @@
       </c>
       <c r="F7" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E7+M7+N7+Y7+AA7+L7</f>
-        <v>1327605.71</v>
+        <v>1327604.97</v>
       </c>
       <c r="G7" s="2" t="n">
         <f aca="false">D7-F7</f>
-        <v>-48885.8399999996</v>
+        <v>-48885.0999999996</v>
       </c>
       <c r="H7" s="3" t="n">
         <f aca="false">ROUND(G7/D7,4)</f>
@@ -6208,15 +6208,15 @@
       </c>
       <c r="Z7" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C7/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA7" s="2" t="n">
         <f aca="false">Z7+O7</f>
-        <v>18381.72</v>
+        <v>18380.98</v>
       </c>
       <c r="AB7" s="2" t="n">
         <f aca="false">F7-L7-S7</f>
-        <v>342125.4</v>
+        <v>342124.66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6239,11 +6239,11 @@
       </c>
       <c r="F8" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E8+M8+N8+Y8+AA8+L8</f>
-        <v>1355760.27</v>
+        <v>1355759.9</v>
       </c>
       <c r="G8" s="2" t="n">
         <f aca="false">D8-F8</f>
-        <v>-77040.3999999999</v>
+        <v>-77040.0299999998</v>
       </c>
       <c r="H8" s="3" t="n">
         <f aca="false">ROUND(G8/D8,4)</f>
@@ -6319,15 +6319,15 @@
       </c>
       <c r="Z8" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C8/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA8" s="2" t="n">
         <f aca="false">Z8+O8</f>
-        <v>9642.3</v>
+        <v>9641.93</v>
       </c>
       <c r="AB8" s="2" t="n">
         <f aca="false">F8-L8-S8</f>
-        <v>313940.25</v>
+        <v>313939.88</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6350,11 +6350,11 @@
       </c>
       <c r="F9" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E9+M9+N9+Y9+AA9+L9</f>
-        <v>1379842.32</v>
+        <v>1379841.77</v>
       </c>
       <c r="G9" s="2" t="n">
         <f aca="false">D9-F9</f>
-        <v>-101122.45</v>
+        <v>-101121.9</v>
       </c>
       <c r="H9" s="3" t="n">
         <f aca="false">ROUND(G9/D9,4)</f>
@@ -6430,15 +6430,15 @@
       </c>
       <c r="Z9" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C9/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA9" s="2" t="n">
         <f aca="false">Z9+O9</f>
-        <v>14463.45</v>
+        <v>14462.9</v>
       </c>
       <c r="AB9" s="2" t="n">
         <f aca="false">F9-L9-S9</f>
-        <v>338022.3</v>
+        <v>338021.75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6461,11 +6461,11 @@
       </c>
       <c r="F10" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E10+M10+N10+Y10+AA10+L10</f>
-        <v>1403924.37</v>
+        <v>1403923.63</v>
       </c>
       <c r="G10" s="2" t="n">
         <f aca="false">D10-F10</f>
-        <v>-125204.5</v>
+        <v>-125203.76</v>
       </c>
       <c r="H10" s="3" t="n">
         <f aca="false">ROUND(G10/D10,4)</f>
@@ -6541,15 +6541,15 @@
       </c>
       <c r="Z10" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C10/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA10" s="2" t="n">
         <f aca="false">Z10+O10</f>
-        <v>19284.6</v>
+        <v>19283.86</v>
       </c>
       <c r="AB10" s="2" t="n">
         <f aca="false">F10-L10-S10</f>
-        <v>362104.35</v>
+        <v>362103.61</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6572,11 +6572,11 @@
       </c>
       <c r="F11" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E11+M11+N11+Y11+AA11+L11</f>
-        <v>1429695.3</v>
+        <v>1429694.93</v>
       </c>
       <c r="G11" s="2" t="n">
         <f aca="false">D11-F11</f>
-        <v>-150975.43</v>
+        <v>-150975.06</v>
       </c>
       <c r="H11" s="3" t="n">
         <f aca="false">ROUND(G11/D11,4)</f>
@@ -6652,15 +6652,15 @@
       </c>
       <c r="Z11" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C11/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA11" s="2" t="n">
         <f aca="false">Z11+O11</f>
-        <v>10093.74</v>
+        <v>10093.37</v>
       </c>
       <c r="AB11" s="2" t="n">
         <f aca="false">F11-L11-S11</f>
-        <v>331535.57</v>
+        <v>331535.2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6683,11 +6683,11 @@
       </c>
       <c r="F12" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E12+M12+N12+Y12+AA12+L12</f>
-        <v>1454969.15</v>
+        <v>1454968.6</v>
       </c>
       <c r="G12" s="2" t="n">
         <f aca="false">D12-F12</f>
-        <v>-176249.28</v>
+        <v>-176248.73</v>
       </c>
       <c r="H12" s="3" t="n">
         <f aca="false">ROUND(G12/D12,4)</f>
@@ -6763,15 +6763,15 @@
       </c>
       <c r="Z12" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C12/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA12" s="2" t="n">
         <f aca="false">Z12+O12</f>
-        <v>15140.61</v>
+        <v>15140.06</v>
       </c>
       <c r="AB12" s="2" t="n">
         <f aca="false">F12-L12-S12</f>
-        <v>356809.42</v>
+        <v>356808.87</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6794,11 +6794,11 @@
       </c>
       <c r="F13" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E13+M13+N13+Y13+AA13+L13</f>
-        <v>1480243</v>
+        <v>1480242.26</v>
       </c>
       <c r="G13" s="2" t="n">
         <f aca="false">D13-F13</f>
-        <v>-201523.13</v>
+        <v>-201522.39</v>
       </c>
       <c r="H13" s="3" t="n">
         <f aca="false">ROUND(G13/D13,4)</f>
@@ -6874,15 +6874,15 @@
       </c>
       <c r="Z13" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C13/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA13" s="2" t="n">
         <f aca="false">Z13+O13</f>
-        <v>20187.48</v>
+        <v>20186.74</v>
       </c>
       <c r="AB13" s="2" t="n">
         <f aca="false">F13-L13-S13</f>
-        <v>382083.27</v>
+        <v>382082.53</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6905,11 +6905,11 @@
       </c>
       <c r="F14" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E14+M14+N14+Y14+AA14+L14</f>
-        <v>1212152.58</v>
+        <v>1212152.21</v>
       </c>
       <c r="G14" s="2" t="n">
         <f aca="false">D14-F14</f>
-        <v>137607.28</v>
+        <v>137607.65</v>
       </c>
       <c r="H14" s="3" t="n">
         <f aca="false">ROUND(G14/D14,4)</f>
@@ -6985,15 +6985,15 @@
       </c>
       <c r="Z14" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C14/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA14" s="2" t="n">
         <f aca="false">Z14+O14</f>
-        <v>8739.42</v>
+        <v>8739.05</v>
       </c>
       <c r="AB14" s="2" t="n">
         <f aca="false">F14-L14-S14</f>
-        <v>278749.58</v>
+        <v>278749.21</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7016,11 +7016,11 @@
       </c>
       <c r="F15" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E15+M15+N15+Y15+AA15+L15</f>
-        <v>1233851.03</v>
+        <v>1233850.48</v>
       </c>
       <c r="G15" s="2" t="n">
         <f aca="false">D15-F15</f>
-        <v>115908.83</v>
+        <v>115909.38</v>
       </c>
       <c r="H15" s="3" t="n">
         <f aca="false">ROUND(G15/D15,4)</f>
@@ -7096,15 +7096,15 @@
       </c>
       <c r="Z15" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C15/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA15" s="2" t="n">
         <f aca="false">Z15+O15</f>
-        <v>13109.13</v>
+        <v>13108.58</v>
       </c>
       <c r="AB15" s="2" t="n">
         <f aca="false">F15-L15-S15</f>
-        <v>300448.03</v>
+        <v>300447.48</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7127,11 +7127,11 @@
       </c>
       <c r="F16" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E16+M16+N16+Y16+AA16+L16</f>
-        <v>1255549.48</v>
+        <v>1255548.74</v>
       </c>
       <c r="G16" s="2" t="n">
         <f aca="false">D16-F16</f>
-        <v>94210.3799999999</v>
+        <v>94211.1199999999</v>
       </c>
       <c r="H16" s="3" t="n">
         <f aca="false">ROUND(G16/D16,4)</f>
@@ -7207,15 +7207,15 @@
       </c>
       <c r="Z16" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C16/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA16" s="2" t="n">
         <f aca="false">Z16+O16</f>
-        <v>17478.84</v>
+        <v>17478.1</v>
       </c>
       <c r="AB16" s="2" t="n">
         <f aca="false">F16-L16-S16</f>
-        <v>322146.48</v>
+        <v>322145.74</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7238,11 +7238,11 @@
       </c>
       <c r="F17" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E17+M17+N17+Y17+AA17+L17</f>
-        <v>1286087.63</v>
+        <v>1286087.26</v>
       </c>
       <c r="G17" s="2" t="n">
         <f aca="false">D17-F17</f>
-        <v>63672.23</v>
+        <v>63672.6000000001</v>
       </c>
       <c r="H17" s="3" t="n">
         <f aca="false">ROUND(G17/D17,4)</f>
@@ -7318,15 +7318,15 @@
       </c>
       <c r="Z17" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C17/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA17" s="2" t="n">
         <f aca="false">Z17+O17</f>
-        <v>9190.86</v>
+        <v>9190.49</v>
       </c>
       <c r="AB17" s="2" t="n">
         <f aca="false">F17-L17-S17</f>
-        <v>296344.92</v>
+        <v>296344.55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7349,11 +7349,11 @@
       </c>
       <c r="F18" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E18+M18+N18+Y18+AA18+L18</f>
-        <v>1308977.86</v>
+        <v>1308977.31</v>
       </c>
       <c r="G18" s="2" t="n">
         <f aca="false">D18-F18</f>
-        <v>40782</v>
+        <v>40782.5500000001</v>
       </c>
       <c r="H18" s="3" t="n">
         <f aca="false">ROUND(G18/D18,4)</f>
@@ -7361,7 +7361,7 @@
       </c>
       <c r="I18" s="3" t="n">
         <f aca="false">IF(AB18&lt;=0,"",ROUND(G18/AB18,4))</f>
-        <v>0.1277</v>
+        <v>0.1278</v>
       </c>
       <c r="J18" s="2" t="n">
         <f aca="false">ROUND(D18*Assumptions!$B$18/100,2)</f>
@@ -7429,15 +7429,15 @@
       </c>
       <c r="Z18" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C18/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA18" s="2" t="n">
         <f aca="false">Z18+O18</f>
-        <v>13786.29</v>
+        <v>13785.74</v>
       </c>
       <c r="AB18" s="2" t="n">
         <f aca="false">F18-L18-S18</f>
-        <v>319235.15</v>
+        <v>319234.6</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7460,11 +7460,11 @@
       </c>
       <c r="F19" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E19+M19+N19+Y19+AA19+L19</f>
-        <v>1331868.11</v>
+        <v>1331867.37</v>
       </c>
       <c r="G19" s="2" t="n">
         <f aca="false">D19-F19</f>
-        <v>17891.7500000002</v>
+        <v>17892.4900000002</v>
       </c>
       <c r="H19" s="3" t="n">
         <f aca="false">ROUND(G19/D19,4)</f>
@@ -7540,15 +7540,15 @@
       </c>
       <c r="Z19" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C19/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA19" s="2" t="n">
         <f aca="false">Z19+O19</f>
-        <v>18381.72</v>
+        <v>18380.98</v>
       </c>
       <c r="AB19" s="2" t="n">
         <f aca="false">F19-L19-S19</f>
-        <v>342125.4</v>
+        <v>342124.66</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7571,11 +7571,11 @@
       </c>
       <c r="F20" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E20+M20+N20+Y20+AA20+L20</f>
-        <v>1360022.67</v>
+        <v>1360022.3</v>
       </c>
       <c r="G20" s="2" t="n">
         <f aca="false">D20-F20</f>
-        <v>-10262.8100000001</v>
+        <v>-10262.4399999999</v>
       </c>
       <c r="H20" s="3" t="n">
         <f aca="false">ROUND(G20/D20,4)</f>
@@ -7651,15 +7651,15 @@
       </c>
       <c r="Z20" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C20/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA20" s="2" t="n">
         <f aca="false">Z20+O20</f>
-        <v>9642.3</v>
+        <v>9641.93</v>
       </c>
       <c r="AB20" s="2" t="n">
         <f aca="false">F20-L20-S20</f>
-        <v>313940.25</v>
+        <v>313939.88</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7682,11 +7682,11 @@
       </c>
       <c r="F21" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E21+M21+N21+Y21+AA21+L21</f>
-        <v>1384104.72</v>
+        <v>1384104.17</v>
       </c>
       <c r="G21" s="2" t="n">
         <f aca="false">D21-F21</f>
-        <v>-34344.8599999999</v>
+        <v>-34344.3099999998</v>
       </c>
       <c r="H21" s="3" t="n">
         <f aca="false">ROUND(G21/D21,4)</f>
@@ -7762,15 +7762,15 @@
       </c>
       <c r="Z21" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C21/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA21" s="2" t="n">
         <f aca="false">Z21+O21</f>
-        <v>14463.45</v>
+        <v>14462.9</v>
       </c>
       <c r="AB21" s="2" t="n">
         <f aca="false">F21-L21-S21</f>
-        <v>338022.3</v>
+        <v>338021.75</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7793,11 +7793,11 @@
       </c>
       <c r="F22" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E22+M22+N22+Y22+AA22+L22</f>
-        <v>1408186.77</v>
+        <v>1408186.03</v>
       </c>
       <c r="G22" s="2" t="n">
         <f aca="false">D22-F22</f>
-        <v>-58426.9100000002</v>
+        <v>-58426.1700000002</v>
       </c>
       <c r="H22" s="3" t="n">
         <f aca="false">ROUND(G22/D22,4)</f>
@@ -7873,15 +7873,15 @@
       </c>
       <c r="Z22" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C22/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA22" s="2" t="n">
         <f aca="false">Z22+O22</f>
-        <v>19284.6</v>
+        <v>19283.86</v>
       </c>
       <c r="AB22" s="2" t="n">
         <f aca="false">F22-L22-S22</f>
-        <v>362104.35</v>
+        <v>362103.61</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7904,11 +7904,11 @@
       </c>
       <c r="F23" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E23+M23+N23+Y23+AA23+L23</f>
-        <v>1433957.7</v>
+        <v>1433957.33</v>
       </c>
       <c r="G23" s="2" t="n">
         <f aca="false">D23-F23</f>
-        <v>-84197.8399999999</v>
+        <v>-84197.47</v>
       </c>
       <c r="H23" s="3" t="n">
         <f aca="false">ROUND(G23/D23,4)</f>
@@ -7984,15 +7984,15 @@
       </c>
       <c r="Z23" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C23/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA23" s="2" t="n">
         <f aca="false">Z23+O23</f>
-        <v>10093.74</v>
+        <v>10093.37</v>
       </c>
       <c r="AB23" s="2" t="n">
         <f aca="false">F23-L23-S23</f>
-        <v>331535.57</v>
+        <v>331535.2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8015,11 +8015,11 @@
       </c>
       <c r="F24" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E24+M24+N24+Y24+AA24+L24</f>
-        <v>1459231.55</v>
+        <v>1459231</v>
       </c>
       <c r="G24" s="2" t="n">
         <f aca="false">D24-F24</f>
-        <v>-109471.69</v>
+        <v>-109471.14</v>
       </c>
       <c r="H24" s="3" t="n">
         <f aca="false">ROUND(G24/D24,4)</f>
@@ -8095,15 +8095,15 @@
       </c>
       <c r="Z24" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C24/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA24" s="2" t="n">
         <f aca="false">Z24+O24</f>
-        <v>15140.61</v>
+        <v>15140.06</v>
       </c>
       <c r="AB24" s="2" t="n">
         <f aca="false">F24-L24-S24</f>
-        <v>356809.42</v>
+        <v>356808.87</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8126,11 +8126,11 @@
       </c>
       <c r="F25" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E25+M25+N25+Y25+AA25+L25</f>
-        <v>1484505.4</v>
+        <v>1484504.66</v>
       </c>
       <c r="G25" s="2" t="n">
         <f aca="false">D25-F25</f>
-        <v>-134745.54</v>
+        <v>-134744.8</v>
       </c>
       <c r="H25" s="3" t="n">
         <f aca="false">ROUND(G25/D25,4)</f>
@@ -8206,15 +8206,15 @@
       </c>
       <c r="Z25" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C25/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA25" s="2" t="n">
         <f aca="false">Z25+O25</f>
-        <v>20187.48</v>
+        <v>20186.74</v>
       </c>
       <c r="AB25" s="2" t="n">
         <f aca="false">F25-L25-S25</f>
-        <v>382083.27</v>
+        <v>382082.53</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8237,11 +8237,11 @@
       </c>
       <c r="F26" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E26+M26+N26+Y26+AA26+L26</f>
-        <v>1216414.98</v>
+        <v>1216414.61</v>
       </c>
       <c r="G26" s="2" t="n">
         <f aca="false">D26-F26</f>
-        <v>204384.87</v>
+        <v>204385.24</v>
       </c>
       <c r="H26" s="3" t="n">
         <f aca="false">ROUND(G26/D26,4)</f>
@@ -8317,15 +8317,15 @@
       </c>
       <c r="Z26" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C26/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA26" s="2" t="n">
         <f aca="false">Z26+O26</f>
-        <v>8739.42</v>
+        <v>8739.05</v>
       </c>
       <c r="AB26" s="2" t="n">
         <f aca="false">F26-L26-S26</f>
-        <v>278749.58</v>
+        <v>278749.21</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8348,11 +8348,11 @@
       </c>
       <c r="F27" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E27+M27+N27+Y27+AA27+L27</f>
-        <v>1238113.43</v>
+        <v>1238112.88</v>
       </c>
       <c r="G27" s="2" t="n">
         <f aca="false">D27-F27</f>
-        <v>182686.42</v>
+        <v>182686.97</v>
       </c>
       <c r="H27" s="3" t="n">
         <f aca="false">ROUND(G27/D27,4)</f>
@@ -8428,15 +8428,15 @@
       </c>
       <c r="Z27" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C27/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA27" s="2" t="n">
         <f aca="false">Z27+O27</f>
-        <v>13109.13</v>
+        <v>13108.58</v>
       </c>
       <c r="AB27" s="2" t="n">
         <f aca="false">F27-L27-S27</f>
-        <v>300448.03</v>
+        <v>300447.48</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8459,11 +8459,11 @@
       </c>
       <c r="F28" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E28+M28+N28+Y28+AA28+L28</f>
-        <v>1259811.88</v>
+        <v>1259811.14</v>
       </c>
       <c r="G28" s="2" t="n">
         <f aca="false">D28-F28</f>
-        <v>160987.97</v>
+        <v>160988.71</v>
       </c>
       <c r="H28" s="3" t="n">
         <f aca="false">ROUND(G28/D28,4)</f>
@@ -8539,15 +8539,15 @@
       </c>
       <c r="Z28" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C28/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA28" s="2" t="n">
         <f aca="false">Z28+O28</f>
-        <v>17478.84</v>
+        <v>17478.1</v>
       </c>
       <c r="AB28" s="2" t="n">
         <f aca="false">F28-L28-S28</f>
-        <v>322146.48</v>
+        <v>322145.74</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8570,11 +8570,11 @@
       </c>
       <c r="F29" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E29+M29+N29+Y29+AA29+L29</f>
-        <v>1290350.03</v>
+        <v>1290349.66</v>
       </c>
       <c r="G29" s="2" t="n">
         <f aca="false">D29-F29</f>
-        <v>130449.82</v>
+        <v>130450.19</v>
       </c>
       <c r="H29" s="3" t="n">
         <f aca="false">ROUND(G29/D29,4)</f>
@@ -8650,15 +8650,15 @@
       </c>
       <c r="Z29" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C29/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA29" s="2" t="n">
         <f aca="false">Z29+O29</f>
-        <v>9190.86</v>
+        <v>9190.49</v>
       </c>
       <c r="AB29" s="2" t="n">
         <f aca="false">F29-L29-S29</f>
-        <v>296344.92</v>
+        <v>296344.55</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8681,11 +8681,11 @@
       </c>
       <c r="F30" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E30+M30+N30+Y30+AA30+L30</f>
-        <v>1313240.26</v>
+        <v>1313239.71</v>
       </c>
       <c r="G30" s="2" t="n">
         <f aca="false">D30-F30</f>
-        <v>107559.59</v>
+        <v>107560.14</v>
       </c>
       <c r="H30" s="3" t="n">
         <f aca="false">ROUND(G30/D30,4)</f>
@@ -8761,15 +8761,15 @@
       </c>
       <c r="Z30" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C30/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA30" s="2" t="n">
         <f aca="false">Z30+O30</f>
-        <v>13786.29</v>
+        <v>13785.74</v>
       </c>
       <c r="AB30" s="2" t="n">
         <f aca="false">F30-L30-S30</f>
-        <v>319235.15</v>
+        <v>319234.6</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8792,11 +8792,11 @@
       </c>
       <c r="F31" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E31+M31+N31+Y31+AA31+L31</f>
-        <v>1336130.51</v>
+        <v>1336129.77</v>
       </c>
       <c r="G31" s="2" t="n">
         <f aca="false">D31-F31</f>
-        <v>84669.3400000003</v>
+        <v>84670.0800000003</v>
       </c>
       <c r="H31" s="3" t="n">
         <f aca="false">ROUND(G31/D31,4)</f>
@@ -8872,15 +8872,15 @@
       </c>
       <c r="Z31" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C31/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA31" s="2" t="n">
         <f aca="false">Z31+O31</f>
-        <v>18381.72</v>
+        <v>18380.98</v>
       </c>
       <c r="AB31" s="2" t="n">
         <f aca="false">F31-L31-S31</f>
-        <v>342125.4</v>
+        <v>342124.66</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8903,11 +8903,11 @@
       </c>
       <c r="F32" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E32+M32+N32+Y32+AA32+L32</f>
-        <v>1364285.07</v>
+        <v>1364284.7</v>
       </c>
       <c r="G32" s="2" t="n">
         <f aca="false">D32-F32</f>
-        <v>56514.78</v>
+        <v>56515.1500000001</v>
       </c>
       <c r="H32" s="3" t="n">
         <f aca="false">ROUND(G32/D32,4)</f>
@@ -8983,15 +8983,15 @@
       </c>
       <c r="Z32" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C32/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA32" s="2" t="n">
         <f aca="false">Z32+O32</f>
-        <v>9642.3</v>
+        <v>9641.93</v>
       </c>
       <c r="AB32" s="2" t="n">
         <f aca="false">F32-L32-S32</f>
-        <v>313940.25</v>
+        <v>313939.88</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9014,11 +9014,11 @@
       </c>
       <c r="F33" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E33+M33+N33+Y33+AA33+L33</f>
-        <v>1388367.12</v>
+        <v>1388366.57</v>
       </c>
       <c r="G33" s="2" t="n">
         <f aca="false">D33-F33</f>
-        <v>32432.7300000002</v>
+        <v>32433.2800000003</v>
       </c>
       <c r="H33" s="3" t="n">
         <f aca="false">ROUND(G33/D33,4)</f>
@@ -9026,7 +9026,7 @@
       </c>
       <c r="I33" s="3" t="n">
         <f aca="false">IF(AB33&lt;=0,"",ROUND(G33/AB33,4))</f>
-        <v>0.0959</v>
+        <v>0.096</v>
       </c>
       <c r="J33" s="2" t="n">
         <f aca="false">ROUND(D33*Assumptions!$B$18/100,2)</f>
@@ -9094,15 +9094,15 @@
       </c>
       <c r="Z33" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C33/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA33" s="2" t="n">
         <f aca="false">Z33+O33</f>
-        <v>14463.45</v>
+        <v>14462.9</v>
       </c>
       <c r="AB33" s="2" t="n">
         <f aca="false">F33-L33-S33</f>
-        <v>338022.3</v>
+        <v>338021.75</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9125,11 +9125,11 @@
       </c>
       <c r="F34" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E34+M34+N34+Y34+AA34+L34</f>
-        <v>1412449.17</v>
+        <v>1412448.43</v>
       </c>
       <c r="G34" s="2" t="n">
         <f aca="false">D34-F34</f>
-        <v>8350.67999999994</v>
+        <v>8351.41999999993</v>
       </c>
       <c r="H34" s="3" t="n">
         <f aca="false">ROUND(G34/D34,4)</f>
@@ -9205,15 +9205,15 @@
       </c>
       <c r="Z34" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C34/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA34" s="2" t="n">
         <f aca="false">Z34+O34</f>
-        <v>19284.6</v>
+        <v>19283.86</v>
       </c>
       <c r="AB34" s="2" t="n">
         <f aca="false">F34-L34-S34</f>
-        <v>362104.35</v>
+        <v>362103.61</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9236,11 +9236,11 @@
       </c>
       <c r="F35" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E35+M35+N35+Y35+AA35+L35</f>
-        <v>1438220.1</v>
+        <v>1438219.73</v>
       </c>
       <c r="G35" s="2" t="n">
         <f aca="false">D35-F35</f>
-        <v>-17420.2499999998</v>
+        <v>-17419.8799999999</v>
       </c>
       <c r="H35" s="3" t="n">
         <f aca="false">ROUND(G35/D35,4)</f>
@@ -9316,15 +9316,15 @@
       </c>
       <c r="Z35" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C35/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA35" s="2" t="n">
         <f aca="false">Z35+O35</f>
-        <v>10093.74</v>
+        <v>10093.37</v>
       </c>
       <c r="AB35" s="2" t="n">
         <f aca="false">F35-L35-S35</f>
-        <v>331535.57</v>
+        <v>331535.2</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9347,11 +9347,11 @@
       </c>
       <c r="F36" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E36+M36+N36+Y36+AA36+L36</f>
-        <v>1463493.95</v>
+        <v>1463493.4</v>
       </c>
       <c r="G36" s="2" t="n">
         <f aca="false">D36-F36</f>
-        <v>-42694.0999999999</v>
+        <v>-42693.5499999998</v>
       </c>
       <c r="H36" s="3" t="n">
         <f aca="false">ROUND(G36/D36,4)</f>
@@ -9427,15 +9427,15 @@
       </c>
       <c r="Z36" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C36/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA36" s="2" t="n">
         <f aca="false">Z36+O36</f>
-        <v>15140.61</v>
+        <v>15140.06</v>
       </c>
       <c r="AB36" s="2" t="n">
         <f aca="false">F36-L36-S36</f>
-        <v>356809.42</v>
+        <v>356808.87</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9458,11 +9458,11 @@
       </c>
       <c r="F37" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E37+M37+N37+Y37+AA37+L37</f>
-        <v>1488767.8</v>
+        <v>1488767.06</v>
       </c>
       <c r="G37" s="2" t="n">
         <f aca="false">D37-F37</f>
-        <v>-67967.9499999997</v>
+        <v>-67967.2099999997</v>
       </c>
       <c r="H37" s="3" t="n">
         <f aca="false">ROUND(G37/D37,4)</f>
@@ -9538,15 +9538,15 @@
       </c>
       <c r="Z37" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C37/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA37" s="2" t="n">
         <f aca="false">Z37+O37</f>
-        <v>20187.48</v>
+        <v>20186.74</v>
       </c>
       <c r="AB37" s="2" t="n">
         <f aca="false">F37-L37-S37</f>
-        <v>382083.27</v>
+        <v>382082.53</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9569,11 +9569,11 @@
       </c>
       <c r="F38" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E38+M38+N38+Y38+AA38+L38</f>
-        <v>1220677.38</v>
+        <v>1220677.01</v>
       </c>
       <c r="G38" s="2" t="n">
         <f aca="false">D38-F38</f>
-        <v>271162.46</v>
+        <v>271162.83</v>
       </c>
       <c r="H38" s="3" t="n">
         <f aca="false">ROUND(G38/D38,4)</f>
@@ -9649,15 +9649,15 @@
       </c>
       <c r="Z38" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C38/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA38" s="2" t="n">
         <f aca="false">Z38+O38</f>
-        <v>8739.42</v>
+        <v>8739.05</v>
       </c>
       <c r="AB38" s="2" t="n">
         <f aca="false">F38-L38-S38</f>
-        <v>278749.58</v>
+        <v>278749.21</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9680,11 +9680,11 @@
       </c>
       <c r="F39" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E39+M39+N39+Y39+AA39+L39</f>
-        <v>1242375.83</v>
+        <v>1242375.28</v>
       </c>
       <c r="G39" s="2" t="n">
         <f aca="false">D39-F39</f>
-        <v>249464.01</v>
+        <v>249464.56</v>
       </c>
       <c r="H39" s="3" t="n">
         <f aca="false">ROUND(G39/D39,4)</f>
@@ -9760,15 +9760,15 @@
       </c>
       <c r="Z39" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C39/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA39" s="2" t="n">
         <f aca="false">Z39+O39</f>
-        <v>13109.13</v>
+        <v>13108.58</v>
       </c>
       <c r="AB39" s="2" t="n">
         <f aca="false">F39-L39-S39</f>
-        <v>300448.03</v>
+        <v>300447.48</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9791,11 +9791,11 @@
       </c>
       <c r="F40" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E40+M40+N40+Y40+AA40+L40</f>
-        <v>1264074.28</v>
+        <v>1264073.54</v>
       </c>
       <c r="G40" s="2" t="n">
         <f aca="false">D40-F40</f>
-        <v>227765.56</v>
+        <v>227766.3</v>
       </c>
       <c r="H40" s="3" t="n">
         <f aca="false">ROUND(G40/D40,4)</f>
@@ -9871,15 +9871,15 @@
       </c>
       <c r="Z40" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C40/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA40" s="2" t="n">
         <f aca="false">Z40+O40</f>
-        <v>17478.84</v>
+        <v>17478.1</v>
       </c>
       <c r="AB40" s="2" t="n">
         <f aca="false">F40-L40-S40</f>
-        <v>322146.48</v>
+        <v>322145.74</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9902,11 +9902,11 @@
       </c>
       <c r="F41" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E41+M41+N41+Y41+AA41+L41</f>
-        <v>1294612.43</v>
+        <v>1294612.06</v>
       </c>
       <c r="G41" s="2" t="n">
         <f aca="false">D41-F41</f>
-        <v>197227.41</v>
+        <v>197227.78</v>
       </c>
       <c r="H41" s="3" t="n">
         <f aca="false">ROUND(G41/D41,4)</f>
@@ -9982,15 +9982,15 @@
       </c>
       <c r="Z41" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C41/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA41" s="2" t="n">
         <f aca="false">Z41+O41</f>
-        <v>9190.86</v>
+        <v>9190.49</v>
       </c>
       <c r="AB41" s="2" t="n">
         <f aca="false">F41-L41-S41</f>
-        <v>296344.92</v>
+        <v>296344.55</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10013,11 +10013,11 @@
       </c>
       <c r="F42" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E42+M42+N42+Y42+AA42+L42</f>
-        <v>1317502.66</v>
+        <v>1317502.11</v>
       </c>
       <c r="G42" s="2" t="n">
         <f aca="false">D42-F42</f>
-        <v>174337.18</v>
+        <v>174337.73</v>
       </c>
       <c r="H42" s="3" t="n">
         <f aca="false">ROUND(G42/D42,4)</f>
@@ -10093,15 +10093,15 @@
       </c>
       <c r="Z42" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C42/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA42" s="2" t="n">
         <f aca="false">Z42+O42</f>
-        <v>13786.29</v>
+        <v>13785.74</v>
       </c>
       <c r="AB42" s="2" t="n">
         <f aca="false">F42-L42-S42</f>
-        <v>319235.15</v>
+        <v>319234.6</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10124,11 +10124,11 @@
       </c>
       <c r="F43" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E43+M43+N43+Y43+AA43+L43</f>
-        <v>1340392.91</v>
+        <v>1340392.17</v>
       </c>
       <c r="G43" s="2" t="n">
         <f aca="false">D43-F43</f>
-        <v>151446.93</v>
+        <v>151447.67</v>
       </c>
       <c r="H43" s="3" t="n">
         <f aca="false">ROUND(G43/D43,4)</f>
@@ -10204,15 +10204,15 @@
       </c>
       <c r="Z43" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C43/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA43" s="2" t="n">
         <f aca="false">Z43+O43</f>
-        <v>18381.72</v>
+        <v>18380.98</v>
       </c>
       <c r="AB43" s="2" t="n">
         <f aca="false">F43-L43-S43</f>
-        <v>342125.4</v>
+        <v>342124.66</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10235,11 +10235,11 @@
       </c>
       <c r="F44" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E44+M44+N44+Y44+AA44+L44</f>
-        <v>1368547.47</v>
+        <v>1368547.1</v>
       </c>
       <c r="G44" s="2" t="n">
         <f aca="false">D44-F44</f>
-        <v>123292.37</v>
+        <v>123292.74</v>
       </c>
       <c r="H44" s="3" t="n">
         <f aca="false">ROUND(G44/D44,4)</f>
@@ -10315,15 +10315,15 @@
       </c>
       <c r="Z44" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C44/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA44" s="2" t="n">
         <f aca="false">Z44+O44</f>
-        <v>9642.3</v>
+        <v>9641.93</v>
       </c>
       <c r="AB44" s="2" t="n">
         <f aca="false">F44-L44-S44</f>
-        <v>313940.25</v>
+        <v>313939.88</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10346,11 +10346,11 @@
       </c>
       <c r="F45" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E45+M45+N45+Y45+AA45+L45</f>
-        <v>1392629.52</v>
+        <v>1392628.97</v>
       </c>
       <c r="G45" s="2" t="n">
         <f aca="false">D45-F45</f>
-        <v>99210.3200000003</v>
+        <v>99210.8700000003</v>
       </c>
       <c r="H45" s="3" t="n">
         <f aca="false">ROUND(G45/D45,4)</f>
@@ -10426,15 +10426,15 @@
       </c>
       <c r="Z45" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C45/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA45" s="2" t="n">
         <f aca="false">Z45+O45</f>
-        <v>14463.45</v>
+        <v>14462.9</v>
       </c>
       <c r="AB45" s="2" t="n">
         <f aca="false">F45-L45-S45</f>
-        <v>338022.3</v>
+        <v>338021.75</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10457,11 +10457,11 @@
       </c>
       <c r="F46" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E46+M46+N46+Y46+AA46+L46</f>
-        <v>1416711.57</v>
+        <v>1416710.83</v>
       </c>
       <c r="G46" s="2" t="n">
         <f aca="false">D46-F46</f>
-        <v>75128.27</v>
+        <v>75129.01</v>
       </c>
       <c r="H46" s="3" t="n">
         <f aca="false">ROUND(G46/D46,4)</f>
@@ -10537,15 +10537,15 @@
       </c>
       <c r="Z46" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C46/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA46" s="2" t="n">
         <f aca="false">Z46+O46</f>
-        <v>19284.6</v>
+        <v>19283.86</v>
       </c>
       <c r="AB46" s="2" t="n">
         <f aca="false">F46-L46-S46</f>
-        <v>362104.35</v>
+        <v>362103.61</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10568,11 +10568,11 @@
       </c>
       <c r="F47" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E47+M47+N47+Y47+AA47+L47</f>
-        <v>1442482.5</v>
+        <v>1442482.13</v>
       </c>
       <c r="G47" s="2" t="n">
         <f aca="false">D47-F47</f>
-        <v>49357.3400000003</v>
+        <v>49357.7100000002</v>
       </c>
       <c r="H47" s="3" t="n">
         <f aca="false">ROUND(G47/D47,4)</f>
@@ -10648,15 +10648,15 @@
       </c>
       <c r="Z47" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C47/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA47" s="2" t="n">
         <f aca="false">Z47+O47</f>
-        <v>10093.74</v>
+        <v>10093.37</v>
       </c>
       <c r="AB47" s="2" t="n">
         <f aca="false">F47-L47-S47</f>
-        <v>331535.57</v>
+        <v>331535.2</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10679,11 +10679,11 @@
       </c>
       <c r="F48" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E48+M48+N48+Y48+AA48+L48</f>
-        <v>1467756.35</v>
+        <v>1467755.8</v>
       </c>
       <c r="G48" s="2" t="n">
         <f aca="false">D48-F48</f>
-        <v>24083.4900000002</v>
+        <v>24084.0400000003</v>
       </c>
       <c r="H48" s="3" t="n">
         <f aca="false">ROUND(G48/D48,4)</f>
@@ -10759,15 +10759,15 @@
       </c>
       <c r="Z48" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C48/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA48" s="2" t="n">
         <f aca="false">Z48+O48</f>
-        <v>15140.61</v>
+        <v>15140.06</v>
       </c>
       <c r="AB48" s="2" t="n">
         <f aca="false">F48-L48-S48</f>
-        <v>356809.42</v>
+        <v>356808.87</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10790,11 +10790,11 @@
       </c>
       <c r="F49" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E49+M49+N49+Y49+AA49+L49</f>
-        <v>1493030.2</v>
+        <v>1493029.46</v>
       </c>
       <c r="G49" s="2" t="n">
         <f aca="false">D49-F49</f>
-        <v>-1190.35999999964</v>
+        <v>-1189.61999999965</v>
       </c>
       <c r="H49" s="3" t="n">
         <f aca="false">ROUND(G49/D49,4)</f>
@@ -10870,15 +10870,15 @@
       </c>
       <c r="Z49" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C49/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA49" s="2" t="n">
         <f aca="false">Z49+O49</f>
-        <v>20187.48</v>
+        <v>20186.74</v>
       </c>
       <c r="AB49" s="2" t="n">
         <f aca="false">F49-L49-S49</f>
-        <v>382083.27</v>
+        <v>382082.53</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10901,11 +10901,11 @@
       </c>
       <c r="F50" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E50+M50+N50+Y50+AA50+L50</f>
-        <v>1224939.78</v>
+        <v>1224939.41</v>
       </c>
       <c r="G50" s="2" t="n">
         <f aca="false">D50-F50</f>
-        <v>337940.06</v>
+        <v>337940.43</v>
       </c>
       <c r="H50" s="3" t="n">
         <f aca="false">ROUND(G50/D50,4)</f>
@@ -10981,15 +10981,15 @@
       </c>
       <c r="Z50" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C50/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA50" s="2" t="n">
         <f aca="false">Z50+O50</f>
-        <v>8739.42</v>
+        <v>8739.05</v>
       </c>
       <c r="AB50" s="2" t="n">
         <f aca="false">F50-L50-S50</f>
-        <v>278749.58</v>
+        <v>278749.21</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11012,11 +11012,11 @@
       </c>
       <c r="F51" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E51+M51+N51+Y51+AA51+L51</f>
-        <v>1246638.23</v>
+        <v>1246637.68</v>
       </c>
       <c r="G51" s="2" t="n">
         <f aca="false">D51-F51</f>
-        <v>316241.61</v>
+        <v>316242.16</v>
       </c>
       <c r="H51" s="3" t="n">
         <f aca="false">ROUND(G51/D51,4)</f>
@@ -11092,15 +11092,15 @@
       </c>
       <c r="Z51" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C51/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA51" s="2" t="n">
         <f aca="false">Z51+O51</f>
-        <v>13109.13</v>
+        <v>13108.58</v>
       </c>
       <c r="AB51" s="2" t="n">
         <f aca="false">F51-L51-S51</f>
-        <v>300448.03</v>
+        <v>300447.48</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11123,11 +11123,11 @@
       </c>
       <c r="F52" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E52+M52+N52+Y52+AA52+L52</f>
-        <v>1268336.68</v>
+        <v>1268335.94</v>
       </c>
       <c r="G52" s="2" t="n">
         <f aca="false">D52-F52</f>
-        <v>294543.16</v>
+        <v>294543.9</v>
       </c>
       <c r="H52" s="3" t="n">
         <f aca="false">ROUND(G52/D52,4)</f>
@@ -11203,15 +11203,15 @@
       </c>
       <c r="Z52" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C52/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA52" s="2" t="n">
         <f aca="false">Z52+O52</f>
-        <v>17478.84</v>
+        <v>17478.1</v>
       </c>
       <c r="AB52" s="2" t="n">
         <f aca="false">F52-L52-S52</f>
-        <v>322146.48</v>
+        <v>322145.74</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11234,11 +11234,11 @@
       </c>
       <c r="F53" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E53+M53+N53+Y53+AA53+L53</f>
-        <v>1298874.83</v>
+        <v>1298874.46</v>
       </c>
       <c r="G53" s="2" t="n">
         <f aca="false">D53-F53</f>
-        <v>264005.01</v>
+        <v>264005.38</v>
       </c>
       <c r="H53" s="3" t="n">
         <f aca="false">ROUND(G53/D53,4)</f>
@@ -11314,15 +11314,15 @@
       </c>
       <c r="Z53" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C53/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA53" s="2" t="n">
         <f aca="false">Z53+O53</f>
-        <v>9190.86</v>
+        <v>9190.49</v>
       </c>
       <c r="AB53" s="2" t="n">
         <f aca="false">F53-L53-S53</f>
-        <v>296344.92</v>
+        <v>296344.55</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11345,11 +11345,11 @@
       </c>
       <c r="F54" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E54+M54+N54+Y54+AA54+L54</f>
-        <v>1321765.06</v>
+        <v>1321764.51</v>
       </c>
       <c r="G54" s="2" t="n">
         <f aca="false">D54-F54</f>
-        <v>241114.78</v>
+        <v>241115.33</v>
       </c>
       <c r="H54" s="3" t="n">
         <f aca="false">ROUND(G54/D54,4)</f>
@@ -11425,15 +11425,15 @@
       </c>
       <c r="Z54" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C54/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA54" s="2" t="n">
         <f aca="false">Z54+O54</f>
-        <v>13786.29</v>
+        <v>13785.74</v>
       </c>
       <c r="AB54" s="2" t="n">
         <f aca="false">F54-L54-S54</f>
-        <v>319235.15</v>
+        <v>319234.6</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11456,11 +11456,11 @@
       </c>
       <c r="F55" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E55+M55+N55+Y55+AA55+L55</f>
-        <v>1344655.31</v>
+        <v>1344654.57</v>
       </c>
       <c r="G55" s="2" t="n">
         <f aca="false">D55-F55</f>
-        <v>218224.53</v>
+        <v>218225.27</v>
       </c>
       <c r="H55" s="3" t="n">
         <f aca="false">ROUND(G55/D55,4)</f>
@@ -11468,7 +11468,7 @@
       </c>
       <c r="I55" s="3" t="n">
         <f aca="false">IF(AB55&lt;=0,"",ROUND(G55/AB55,4))</f>
-        <v>0.6378</v>
+        <v>0.6379</v>
       </c>
       <c r="J55" s="2" t="n">
         <f aca="false">ROUND(D55*Assumptions!$B$18/100,2)</f>
@@ -11536,15 +11536,15 @@
       </c>
       <c r="Z55" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C55/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA55" s="2" t="n">
         <f aca="false">Z55+O55</f>
-        <v>18381.72</v>
+        <v>18380.98</v>
       </c>
       <c r="AB55" s="2" t="n">
         <f aca="false">F55-L55-S55</f>
-        <v>342125.4</v>
+        <v>342124.66</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11567,11 +11567,11 @@
       </c>
       <c r="F56" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E56+M56+N56+Y56+AA56+L56</f>
-        <v>1372809.87</v>
+        <v>1372809.5</v>
       </c>
       <c r="G56" s="2" t="n">
         <f aca="false">D56-F56</f>
-        <v>190069.97</v>
+        <v>190070.34</v>
       </c>
       <c r="H56" s="3" t="n">
         <f aca="false">ROUND(G56/D56,4)</f>
@@ -11647,15 +11647,15 @@
       </c>
       <c r="Z56" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C56/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA56" s="2" t="n">
         <f aca="false">Z56+O56</f>
-        <v>9642.3</v>
+        <v>9641.93</v>
       </c>
       <c r="AB56" s="2" t="n">
         <f aca="false">F56-L56-S56</f>
-        <v>313940.25</v>
+        <v>313939.88</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11678,11 +11678,11 @@
       </c>
       <c r="F57" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E57+M57+N57+Y57+AA57+L57</f>
-        <v>1396891.92</v>
+        <v>1396891.37</v>
       </c>
       <c r="G57" s="2" t="n">
         <f aca="false">D57-F57</f>
-        <v>165987.92</v>
+        <v>165988.47</v>
       </c>
       <c r="H57" s="3" t="n">
         <f aca="false">ROUND(G57/D57,4)</f>
@@ -11758,15 +11758,15 @@
       </c>
       <c r="Z57" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C57/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA57" s="2" t="n">
         <f aca="false">Z57+O57</f>
-        <v>14463.45</v>
+        <v>14462.9</v>
       </c>
       <c r="AB57" s="2" t="n">
         <f aca="false">F57-L57-S57</f>
-        <v>338022.3</v>
+        <v>338021.75</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11789,11 +11789,11 @@
       </c>
       <c r="F58" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E58+M58+N58+Y58+AA58+L58</f>
-        <v>1420973.97</v>
+        <v>1420973.23</v>
       </c>
       <c r="G58" s="2" t="n">
         <f aca="false">D58-F58</f>
-        <v>141905.87</v>
+        <v>141906.61</v>
       </c>
       <c r="H58" s="3" t="n">
         <f aca="false">ROUND(G58/D58,4)</f>
@@ -11869,15 +11869,15 @@
       </c>
       <c r="Z58" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C58/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA58" s="2" t="n">
         <f aca="false">Z58+O58</f>
-        <v>19284.6</v>
+        <v>19283.86</v>
       </c>
       <c r="AB58" s="2" t="n">
         <f aca="false">F58-L58-S58</f>
-        <v>362104.35</v>
+        <v>362103.61</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11900,11 +11900,11 @@
       </c>
       <c r="F59" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E59+M59+N59+Y59+AA59+L59</f>
-        <v>1446744.9</v>
+        <v>1446744.53</v>
       </c>
       <c r="G59" s="2" t="n">
         <f aca="false">D59-F59</f>
-        <v>116134.94</v>
+        <v>116135.31</v>
       </c>
       <c r="H59" s="3" t="n">
         <f aca="false">ROUND(G59/D59,4)</f>
@@ -11980,15 +11980,15 @@
       </c>
       <c r="Z59" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C59/12,2)</f>
-        <v>4676.46</v>
+        <v>4676.09</v>
       </c>
       <c r="AA59" s="2" t="n">
         <f aca="false">Z59+O59</f>
-        <v>10093.74</v>
+        <v>10093.37</v>
       </c>
       <c r="AB59" s="2" t="n">
         <f aca="false">F59-L59-S59</f>
-        <v>331535.57</v>
+        <v>331535.2</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12011,11 +12011,11 @@
       </c>
       <c r="F60" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E60+M60+N60+Y60+AA60+L60</f>
-        <v>1472018.75</v>
+        <v>1472018.2</v>
       </c>
       <c r="G60" s="2" t="n">
         <f aca="false">D60-F60</f>
-        <v>90861.0900000001</v>
+        <v>90861.6400000001</v>
       </c>
       <c r="H60" s="3" t="n">
         <f aca="false">ROUND(G60/D60,4)</f>
@@ -12023,7 +12023,7 @@
       </c>
       <c r="I60" s="3" t="n">
         <f aca="false">IF(AB60&lt;=0,"",ROUND(G60/AB60,4))</f>
-        <v>0.2546</v>
+        <v>0.2547</v>
       </c>
       <c r="J60" s="2" t="n">
         <f aca="false">ROUND(D60*Assumptions!$B$18/100,2)</f>
@@ -12091,15 +12091,15 @@
       </c>
       <c r="Z60" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C60/12,2)</f>
-        <v>7014.69</v>
+        <v>7014.14</v>
       </c>
       <c r="AA60" s="2" t="n">
         <f aca="false">Z60+O60</f>
-        <v>15140.61</v>
+        <v>15140.06</v>
       </c>
       <c r="AB60" s="2" t="n">
         <f aca="false">F60-L60-S60</f>
-        <v>356809.42</v>
+        <v>356808.87</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12122,11 +12122,11 @@
       </c>
       <c r="F61" s="2" t="n">
         <f aca="false">S1!$B$2+S1!$B$31+S1!$B$32+E61+M61+N61+Y61+AA61+L61</f>
-        <v>1497292.6</v>
+        <v>1497291.86</v>
       </c>
       <c r="G61" s="2" t="n">
         <f aca="false">D61-F61</f>
-        <v>65587.2400000002</v>
+        <v>65587.9800000002</v>
       </c>
       <c r="H61" s="3" t="n">
         <f aca="false">ROUND(G61/D61,4)</f>
@@ -12202,15 +12202,15 @@
       </c>
       <c r="Z61" s="2" t="n">
         <f aca="false">ROUND(S1!$B$2*Assumptions!$B$16/100*C61/12,2)</f>
-        <v>9352.92</v>
+        <v>9352.18</v>
       </c>
       <c r="AA61" s="2" t="n">
         <f aca="false">Z61+O61</f>
-        <v>20187.48</v>
+        <v>20186.74</v>
       </c>
       <c r="AB61" s="2" t="n">
         <f aca="false">F61-L61-S61</f>
-        <v>382083.27</v>
+        <v>382082.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>